<commit_message>
Added - JOR and CTSR Component in the Project
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7413D766-4D5E-442D-A469-572BA1EF1B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0219DF4C-DC96-4429-8327-F5A96A28C3C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="131">
   <si>
     <t>Name</t>
   </si>
@@ -400,18 +400,12 @@
     <t>JobNumber</t>
   </si>
   <si>
-    <t>DataService_EntityName</t>
-  </si>
-  <si>
     <t>SpectrumJobOverviewReport</t>
   </si>
   <si>
     <t>Field or column name that holds the Job name details in the Entity.</t>
   </si>
   <si>
-    <t>Data Service Name</t>
-  </si>
-  <si>
     <t>Report_Format</t>
   </si>
   <si>
@@ -425,6 +419,21 @@
   </si>
   <si>
     <t>Job Overview Report - Through Period End Date - "dd/MM/YY"</t>
+  </si>
+  <si>
+    <t>DS_JOR_EntityName</t>
+  </si>
+  <si>
+    <t>SpectrumCostTypeSummaryReport</t>
+  </si>
+  <si>
+    <t>DS_CTSR_EntityName</t>
+  </si>
+  <si>
+    <t>Data Service Name for Job Overview Report</t>
+  </si>
+  <si>
+    <t>Data Service Name for Cost Type Summary Report</t>
   </si>
 </sst>
 </file>
@@ -855,7 +864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y27"/>
+  <dimension ref="A1:Y28"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
@@ -1085,57 +1094,68 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>120</v>
-      </c>
       <c r="C22" s="2" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B24" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" t="s">
-        <v>114</v>
-      </c>
-      <c r="B24" t="s">
-        <v>114</v>
-      </c>
       <c r="C24" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>114</v>
+      </c>
+      <c r="B25" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
         <v>116</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B26" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C26" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>121</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C28" t="s">
         <v>123</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="C27" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2436,16 +2456,16 @@
     </row>
     <row r="8" spans="1:25">
       <c r="A8" s="16" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>67</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Added - JOR To BFR, CTSR  and BHR Extraction
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0219DF4C-DC96-4429-8327-F5A96A28C3C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A5661F-91C4-4EA7-8BFD-0DEC80CB45F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="141">
   <si>
     <t>Name</t>
   </si>
@@ -146,12 +146,6 @@
     <t>EmailTo</t>
   </si>
   <si>
-    <t>EmailBcc</t>
-  </si>
-  <si>
-    <t>EmailCc</t>
-  </si>
-  <si>
     <t>EmailSubject</t>
   </si>
   <si>
@@ -179,14 +173,6 @@
     <t>System Exception Occurred</t>
   </si>
   <si>
-    <t>Dear Team,
-Please find the attached Bot status report.
-If you have any further questions or concerns in the meantime, please don’t hesitate to contact us.
-Thank you for your understanding.
-Best regards,
-Support Team</t>
-  </si>
-  <si>
     <t>The delay or time interval before retrying the action for the AP Invoice Mailbox connection.</t>
   </si>
   <si>
@@ -218,9 +204,6 @@
   </si>
   <si>
     <t>Inbox\Spectrum MFA</t>
-  </si>
-  <si>
-    <t>pegasus@inpwrinc.com;calypso@inpwrinc.com;mercury@inpwrinc.com</t>
   </si>
   <si>
     <t>Hi,
@@ -241,9 +224,6 @@
 Support Team</t>
   </si>
   <si>
-    <t>calypso@inpwrinc.com;pegasus@inpwrinc.com;mercury@inpwrinc.com;iris@inpwrinc.com</t>
-  </si>
-  <si>
     <t>Billing/24114 Billing Forecast</t>
   </si>
   <si>
@@ -415,9 +395,6 @@
     <t>Report format to be exported from Spectrum</t>
   </si>
   <si>
-    <t>JOR_EndDate</t>
-  </si>
-  <si>
     <t>Job Overview Report - Through Period End Date - "dd/MM/YY"</t>
   </si>
   <si>
@@ -434,6 +411,63 @@
   </si>
   <si>
     <t>Data Service Name for Cost Type Summary Report</t>
+  </si>
+  <si>
+    <t>JOR_ReportName</t>
+  </si>
+  <si>
+    <t>CTSR_ReportName</t>
+  </si>
+  <si>
+    <t>BHR_ReportName</t>
+  </si>
+  <si>
+    <t>Billing History Report</t>
+  </si>
+  <si>
+    <t>Cost Type Summary Report</t>
+  </si>
+  <si>
+    <t>Job Overview Report</t>
+  </si>
+  <si>
+    <t>BHR_Invoice</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>BHR_Division</t>
+  </si>
+  <si>
+    <t>BHR_From_GL_Date</t>
+  </si>
+  <si>
+    <t>BHR_From_Invoice_Date</t>
+  </si>
+  <si>
+    <t>CurrentMonth_EndDate</t>
+  </si>
+  <si>
+    <t>Dear Automation Team,
+We have successfully processed the Billing forecast for 24114 – CACI CRANE. Attached are the spectrum reports &amp; the updated template for the month &lt;month&gt;
+Please reach out to automationsupport@inpwrinc.com for queries/clarifications.
+Regards,
+Bot</t>
+  </si>
+  <si>
+    <t>Dear Automation Team,
+We have processed the Billing forecast for 24114 – CACI CRANE. Attached are the spectrum reports &amp; the updated template for the Month &lt;Month&gt;. We observed few verification mis-matches as below, 
+&lt;List of all BRES&gt;
+Please reach out to automationsupport@inpwrinc.com for queries/clarifications.
+Regards,
+Bot</t>
+  </si>
+  <si>
+    <t>mercury@inpwrinc.com</t>
+  </si>
+  <si>
+    <t>EM0002</t>
   </si>
 </sst>
 </file>
@@ -502,7 +536,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -522,9 +556,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -539,14 +570,26 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -864,20 +907,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y28"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:Y37"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.28515625" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.42578125" customWidth="1"/>
-    <col min="4" max="25" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="46.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="67.44140625" customWidth="1"/>
+    <col min="4" max="25" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="18.75">
+    <row r="1" spans="1:25" ht="18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -910,110 +953,110 @@
       <c r="A2" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="11" t="s">
-        <v>101</v>
+      <c r="B2" s="10" t="s">
+        <v>96</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:25">
       <c r="A3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" s="10">
+        <v>75</v>
+      </c>
+      <c r="B3" s="9">
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:25">
       <c r="A4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B4" s="10">
+        <v>76</v>
+      </c>
+      <c r="B4" s="9">
         <v>30</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:25">
       <c r="A5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>54</v>
+        <v>77</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:25">
       <c r="A6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>102</v>
+        <v>78</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>97</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:25">
       <c r="A7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>61</v>
+        <v>79</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" t="s">
-        <v>85</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>62</v>
+        <v>80</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" t="s">
-        <v>86</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>74</v>
+        <v>81</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:25">
       <c r="A10" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C10" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C11" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1026,136 +1069,186 @@
     </row>
     <row r="14" spans="1:25">
       <c r="A14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" t="s">
         <v>88</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="C14" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:25">
       <c r="A15" t="s">
-        <v>89</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>91</v>
+        <v>84</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>86</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:25">
       <c r="A16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>95</v>
-      </c>
       <c r="C16" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="C17" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>96</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>67</v>
+        <v>91</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>62</v>
       </c>
       <c r="C18" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>99</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>100</v>
+        <v>94</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>95</v>
       </c>
       <c r="C19" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>98</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>97</v>
+        <v>93</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>114</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>127</v>
+        <v>122</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>121</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>118</v>
+        <v>112</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>113</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B25" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>116</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>74</v>
+        <v>111</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="C26" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>121</v>
-      </c>
-      <c r="B28" s="11" t="s">
-        <v>122</v>
+        <v>116</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>117</v>
       </c>
       <c r="C28" t="s">
-        <v>123</v>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>125</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>126</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>127</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>131</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1168,19 +1261,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
-    <col min="2" max="2" width="51" style="11" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="51" style="10" customWidth="1"/>
+    <col min="3" max="3" width="75.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1210,22 +1303,22 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="28.8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="11">
+      <c r="B2" s="10">
         <v>0</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="10">
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -1237,7 +1330,7 @@
       <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C5" t="s">
@@ -1249,7 +1342,7 @@
       <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>10</v>
       </c>
       <c r="C7" t="s">
@@ -1260,7 +1353,7 @@
       <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>12</v>
       </c>
       <c r="C8" t="s">
@@ -1271,7 +1364,7 @@
       <c r="A9" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C9" t="s">
@@ -1282,7 +1375,7 @@
       <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>17</v>
       </c>
       <c r="C10" t="s">
@@ -1293,7 +1386,7 @@
       <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>19</v>
       </c>
       <c r="C11" t="s">
@@ -1304,7 +1397,7 @@
       <c r="A12" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>37</v>
       </c>
       <c r="C12" t="s">
@@ -1316,7 +1409,7 @@
       <c r="A14" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="10">
         <v>2</v>
       </c>
       <c r="C14" t="s">
@@ -1327,7 +1420,7 @@
       <c r="A15" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="10">
         <v>2</v>
       </c>
       <c r="C15" t="s">
@@ -1335,11 +1428,11 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
+    <row r="17" spans="1:3" ht="28.8">
       <c r="A17" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="11" t="b">
+      <c r="B17" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C17" s="3" t="s">
@@ -2327,12 +2420,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Y969"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="32.85546875" customWidth="1"/>
-    <col min="2" max="2" width="31.140625" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="25" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="32.88671875" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" customWidth="1"/>
+    <col min="3" max="3" width="30.33203125" customWidth="1"/>
+    <col min="4" max="25" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="14.25" customHeight="1">
@@ -2372,100 +2465,100 @@
     </row>
     <row r="2" spans="1:25" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>74</v>
+        <v>63</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>74</v>
+        <v>71</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>67</v>
+        <v>73</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>62</v>
       </c>
       <c r="D4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" t="s">
         <v>67</v>
-      </c>
-      <c r="D5" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="14.25" customHeight="1">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>67</v>
+        <v>64</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:25" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>74</v>
+        <v>108</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25">
-      <c r="A8" s="16" t="s">
-        <v>124</v>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" ht="14.4">
+      <c r="A8" s="14" t="s">
+        <v>136</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>67</v>
+        <v>136</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>62</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1"/>
@@ -3439,73 +3532,73 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A045ED-89B2-46F5-87BB-9D73B35EE197}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="7"/>
+    <col min="4" max="4" width="26.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:5" ht="18">
+      <c r="A1" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="11" customFormat="1" ht="230.4">
+      <c r="A2" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" s="12" customFormat="1" ht="240">
-      <c r="A2" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="210">
-      <c r="A3" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>65</v>
+      <c r="C2" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="201.6">
+      <c r="A3" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="15"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="13"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3514,51 +3607,56 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7C6B43-6EA4-4DD0-939E-D4A6AD374EA2}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="7"/>
+    <col min="3" max="3" width="26.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75">
+    <row r="1" spans="1:4" ht="18">
       <c r="A1" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="150">
+    </row>
+    <row r="2" spans="1:4" ht="158.4">
       <c r="A2" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="12"/>
-      <c r="E2" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="187.2">
+      <c r="A3" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added - BHR and Send email workflow
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A5661F-91C4-4EA7-8BFD-0DEC80CB45F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B15655DF-9A80-43B0-930D-A791696507E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -464,10 +464,10 @@
 Bot</t>
   </si>
   <si>
-    <t>mercury@inpwrinc.com</t>
-  </si>
-  <si>
     <t>EM0002</t>
+  </si>
+  <si>
+    <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
   </si>
 </sst>
 </file>
@@ -536,7 +536,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -576,20 +576,17 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -908,15 +905,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y37"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="46.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.33203125" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.44140625" customWidth="1"/>
-    <col min="4" max="25" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="67.42578125" customWidth="1"/>
+    <col min="4" max="25" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="18">
+    <row r="1" spans="1:25" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1261,12 +1258,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" style="10" customWidth="1"/>
-    <col min="3" max="3" width="75.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col min="3" max="3" width="75.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1303,7 +1300,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="28.8">
+    <row r="2" spans="1:26" ht="30">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1314,7 +1311,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -1428,7 +1425,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="28.8">
+    <row r="17" spans="1:3" ht="45">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -2420,12 +2417,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Y969"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="32.88671875" customWidth="1"/>
-    <col min="2" max="2" width="31.109375" customWidth="1"/>
-    <col min="3" max="3" width="30.33203125" customWidth="1"/>
-    <col min="4" max="25" width="65.44140625" customWidth="1"/>
+    <col min="1" max="1" width="32.85546875" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" customWidth="1"/>
+    <col min="4" max="25" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="14.25" customHeight="1">
@@ -2547,7 +2544,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="14.4">
+    <row r="8" spans="1:25">
       <c r="A8" s="14" t="s">
         <v>136</v>
       </c>
@@ -3532,64 +3529,64 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A045ED-89B2-46F5-87BB-9D73B35EE197}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="7"/>
+    <col min="4" max="4" width="26.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:5" ht="18.75">
+      <c r="A1" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="15" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="11" customFormat="1" ht="230.4">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:5" s="11" customFormat="1" ht="240">
+      <c r="A2" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="16" t="s">
         <v>44</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="D2" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="D2" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="17" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="201.6">
-      <c r="A3" s="17" t="s">
+    <row r="3" spans="1:5" ht="210">
+      <c r="A3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>56</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="D3" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="D3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="17" t="s">
         <v>61</v>
       </c>
     </row>
@@ -3608,16 +3605,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7C6B43-6EA4-4DD0-939E-D4A6AD374EA2}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.109375" style="7"/>
+    <col min="3" max="3" width="26.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18">
+    <row r="1" spans="1:4" ht="18.75">
       <c r="A1" s="6" t="s">
         <v>45</v>
       </c>
@@ -3631,12 +3628,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="158.4">
+    <row r="2" spans="1:4" ht="165">
       <c r="A2" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>139</v>
+      <c r="B2" s="18" t="s">
+        <v>140</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>47</v>
@@ -3645,12 +3642,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="187.2">
+    <row r="3" spans="1:4" ht="210">
       <c r="A3" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>140</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>139</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
updated - updated workflow for year and DS
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B15655DF-9A80-43B0-930D-A791696507E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDC901E-345D-45DD-9040-A1A66F95E18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="143">
   <si>
     <t>Name</t>
   </si>
@@ -468,6 +468,12 @@
   </si>
   <si>
     <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
+  </si>
+  <si>
+    <t>BillingForecastTemplate_DSName</t>
+  </si>
+  <si>
+    <t>BillingForecastTemplateMap</t>
   </si>
 </sst>
 </file>
@@ -585,7 +591,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -904,16 +910,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y37"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:Y38"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.28515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.42578125" customWidth="1"/>
-    <col min="4" max="25" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="46.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="67.44140625" customWidth="1"/>
+    <col min="4" max="25" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="18.75">
+    <row r="1" spans="1:25" ht="18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1132,107 +1138,107 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>123</v>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B25" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>115</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" t="s">
-        <v>109</v>
-      </c>
-      <c r="B25" t="s">
-        <v>109</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" t="s">
+        <v>109</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
         <v>111</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B27" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C27" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
-      <c r="A28" t="s">
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
         <v>116</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B29" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C29" t="s">
         <v>118</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>125</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
+        <v>126</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
         <v>127</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B33" s="10" t="s">
         <v>128</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2">
-      <c r="A34" t="s">
-        <v>131</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>132</v>
@@ -1240,11 +1246,19 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>134</v>
+        <v>133</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
         <v>135</v>
       </c>
     </row>
@@ -1258,12 +1272,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" style="10" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1300,7 +1314,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="28.8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1311,7 +1325,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -1425,7 +1439,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
+    <row r="17" spans="1:3" ht="28.8">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -2417,12 +2431,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Y969"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="32.85546875" customWidth="1"/>
-    <col min="2" max="2" width="31.140625" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="25" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="32.88671875" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" customWidth="1"/>
+    <col min="3" max="3" width="30.33203125" customWidth="1"/>
+    <col min="4" max="25" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="14.25" customHeight="1">
@@ -2544,7 +2558,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:25">
+    <row r="8" spans="1:25" ht="14.4">
       <c r="A8" s="14" t="s">
         <v>136</v>
       </c>
@@ -3529,17 +3543,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A045ED-89B2-46F5-87BB-9D73B35EE197}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="7"/>
+    <col min="4" max="4" width="26.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75">
+    <row r="1" spans="1:5" ht="18">
       <c r="A1" s="15" t="s">
         <v>42</v>
       </c>
@@ -3556,7 +3570,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="11" customFormat="1" ht="240">
+    <row r="2" spans="1:5" s="11" customFormat="1" ht="230.4">
       <c r="A2" s="16" t="s">
         <v>43</v>
       </c>
@@ -3573,7 +3587,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="210">
+    <row r="3" spans="1:5" ht="201.6">
       <c r="A3" s="16" t="s">
         <v>54</v>
       </c>
@@ -3605,16 +3619,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7C6B43-6EA4-4DD0-939E-D4A6AD374EA2}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="7"/>
+    <col min="3" max="3" width="26.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75">
+    <row r="1" spans="1:4" ht="18">
       <c r="A1" s="6" t="s">
         <v>45</v>
       </c>
@@ -3628,7 +3642,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="165">
+    <row r="2" spans="1:4" ht="158.4">
       <c r="A2" s="7" t="s">
         <v>46</v>
       </c>
@@ -3642,7 +3656,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="210">
+    <row r="3" spans="1:4" ht="187.2">
       <c r="A3" s="7" t="s">
         <v>139</v>
       </c>

</xml_diff>

<commit_message>
Added - BHR validation and send email flow with HTML
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://qbotica-my.sharepoint.com/personal/premkumar_sivakumar_qbotica_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDC901E-345D-45DD-9040-A1A66F95E18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="14_{2AA3EA44-538C-46F1-80C7-01D43EBC6AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F6FDDF0-CAC3-4BF4-86C7-E6DBE390082B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="145">
   <si>
     <t>Name</t>
   </si>
@@ -165,9 +165,6 @@
   </si>
   <si>
     <t>EM0001</t>
-  </si>
-  <si>
-    <t>Bot Status Report</t>
   </si>
   <si>
     <t>System Exception Occurred</t>
@@ -449,31 +446,69 @@
     <t>CurrentMonth_EndDate</t>
   </si>
   <si>
-    <t>Dear Automation Team,
-We have successfully processed the Billing forecast for 24114 – CACI CRANE. Attached are the spectrum reports &amp; the updated template for the month &lt;month&gt;
-Please reach out to automationsupport@inpwrinc.com for queries/clarifications.
-Regards,
-Bot</t>
-  </si>
-  <si>
-    <t>Dear Automation Team,
-We have processed the Billing forecast for 24114 – CACI CRANE. Attached are the spectrum reports &amp; the updated template for the Month &lt;Month&gt;. We observed few verification mis-matches as below, 
+    <t>EM0002</t>
+  </si>
+  <si>
+    <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
+  </si>
+  <si>
+    <t>BillingForecastTemplate_DSName</t>
+  </si>
+  <si>
+    <t>BillingForecastTemplateMap</t>
+  </si>
+  <si>
+    <t>mercury@inpwrinc.com</t>
+  </si>
+  <si>
+    <t>Billing forecast for 24114</t>
+  </si>
+  <si>
+    <t>Billing forecast for 24114 with BRE</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;
+ Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have successfully processed the billing forecast for 
+  &lt;strong&gt;24114 – CACI CRANE&lt;/strong&gt;. Attached are the Spectrum reports 
+  and the updated template for the month {0}
+&lt;/p&gt;
+&lt;p&gt;
+  Please reach out to 
+  &lt;a href="mailto:automationsupport@inpwrinc.com"&gt;
+    automationsupport@inpwrinc.com
+  &lt;/a&gt; 
+  for any queries or clarifications.
+&lt;/p&gt;
+&lt;p&gt;
+  Regards,&lt;br/&gt;
+  Bot
+&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;style&gt;
+  table {
+    border-collapse: collapse;
+    border: 1px solid black;
+  }
+  th, td {
+    border: 1px solid black;
+    padding: 8px;
+  }
+&lt;/style&gt;
+&lt;p&gt;
+Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have processed the Billing forecast for &lt;strong&gt;24114 – CACI CRANE&lt;/strong&gt;. Attached are the spectrum reports &amp; the updated template for the Month {0}. &lt;br/&gt;We observed few verification mis-matches as below, 
+&lt;/p&gt;
+&lt;p&gt;Business Rule Excetions: &lt;/p&gt;
+&lt;table&gt;
+&lt;tr&gt;&lt;th&gt;Report Name&lt;/th&gt;&lt;th&gt;Description&lt;/th&gt;&lt;/tr&gt;
 &lt;List of all BRES&gt;
-Please reach out to automationsupport@inpwrinc.com for queries/clarifications.
-Regards,
-Bot</t>
-  </si>
-  <si>
-    <t>EM0002</t>
-  </si>
-  <si>
-    <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
-  </si>
-  <si>
-    <t>BillingForecastTemplate_DSName</t>
-  </si>
-  <si>
-    <t>BillingForecastTemplateMap</t>
+&lt;/table&gt;
+&lt;br/&gt;
+&lt;p&gt;Please reach out to &lt;a href="mailto:automationsupport@inpwrinc.com"&gt; automationsupport@inpwrinc.com &lt;/a&gt; for any queries or clarifications.&lt;/p&gt;
+&lt;p&gt;
+  Regards,&lt;br/&gt;
+  Bot
+&lt;/p&gt;</t>
   </si>
 </sst>
 </file>
@@ -542,7 +577,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -551,12 +586,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -593,6 +622,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -914,7 +946,7 @@
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="46.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.33203125" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="67.44140625" customWidth="1"/>
     <col min="4" max="25" width="8.6640625" customWidth="1"/>
   </cols>
@@ -923,7 +955,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -956,110 +988,110 @@
       <c r="A2" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>96</v>
+      <c r="B2" s="8" t="s">
+        <v>95</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:25">
       <c r="A3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B3" s="9">
+        <v>74</v>
+      </c>
+      <c r="B3" s="7">
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:25">
       <c r="A4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B4" s="9">
+        <v>75</v>
+      </c>
+      <c r="B4" s="7">
         <v>30</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:25">
       <c r="A5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>51</v>
+        <v>76</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:25">
       <c r="A6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B6" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C6" t="s">
         <v>97</v>
-      </c>
-      <c r="C6" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:25">
       <c r="A7" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>58</v>
+        <v>78</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>59</v>
+        <v>79</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>69</v>
+        <v>80</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:25">
       <c r="A10" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1072,194 +1104,194 @@
     </row>
     <row r="14" spans="1:25">
       <c r="A14" t="s">
-        <v>83</v>
-      </c>
-      <c r="B14" s="10" t="s">
         <v>82</v>
       </c>
+      <c r="B14" s="8" t="s">
+        <v>81</v>
+      </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:25">
       <c r="A15" t="s">
-        <v>84</v>
-      </c>
-      <c r="B15" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C15" t="s">
         <v>86</v>
-      </c>
-      <c r="C15" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:25">
       <c r="A16" t="s">
-        <v>85</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>90</v>
+        <v>84</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>89</v>
       </c>
       <c r="C16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="C17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>91</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>62</v>
+        <v>90</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>61</v>
       </c>
       <c r="C18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>95</v>
-      </c>
       <c r="C19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>93</v>
-      </c>
-      <c r="B20" s="10" t="s">
         <v>92</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>141</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>142</v>
+        <v>138</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>114</v>
+        <v>119</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>113</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B24" s="9" t="s">
         <v>121</v>
       </c>
+      <c r="B24" s="7" t="s">
+        <v>120</v>
+      </c>
       <c r="C24" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B25" s="9" t="s">
-        <v>113</v>
-      </c>
       <c r="C25" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="B26" t="s">
-        <v>109</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>111</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>69</v>
+        <v>110</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="C27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
+        <v>115</v>
+      </c>
+      <c r="B29" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="C29" t="s">
         <v>117</v>
-      </c>
-      <c r="C29" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>125</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>130</v>
+        <v>124</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>126</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>129</v>
+        <v>125</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
+        <v>126</v>
+      </c>
+      <c r="B33" s="8" t="s">
         <v>127</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
+        <v>130</v>
+      </c>
+      <c r="B35" s="8" t="s">
         <v>131</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>133</v>
-      </c>
-      <c r="B36" s="10" t="s">
         <v>132</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1275,7 +1307,7 @@
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
-    <col min="2" max="2" width="51" style="10" customWidth="1"/>
+    <col min="2" max="2" width="51" style="8" customWidth="1"/>
     <col min="3" max="3" width="75.44140625" customWidth="1"/>
     <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
@@ -1284,7 +1316,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1318,7 +1350,7 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="8">
         <v>0</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1329,7 +1361,7 @@
       <c r="A3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -1341,7 +1373,7 @@
       <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C5" t="s">
@@ -1353,7 +1385,7 @@
       <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="8" t="s">
         <v>10</v>
       </c>
       <c r="C7" t="s">
@@ -1364,7 +1396,7 @@
       <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="8" t="s">
         <v>12</v>
       </c>
       <c r="C8" t="s">
@@ -1375,7 +1407,7 @@
       <c r="A9" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="8" t="s">
         <v>15</v>
       </c>
       <c r="C9" t="s">
@@ -1386,7 +1418,7 @@
       <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="8" t="s">
         <v>17</v>
       </c>
       <c r="C10" t="s">
@@ -1397,7 +1429,7 @@
       <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C11" t="s">
@@ -1408,7 +1440,7 @@
       <c r="A12" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="8" t="s">
         <v>37</v>
       </c>
       <c r="C12" t="s">
@@ -1420,7 +1452,7 @@
       <c r="A14" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="8">
         <v>2</v>
       </c>
       <c r="C14" t="s">
@@ -1431,7 +1463,7 @@
       <c r="A15" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="8">
         <v>2</v>
       </c>
       <c r="C15" t="s">
@@ -1443,7 +1475,7 @@
       <c r="A17" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="10" t="b">
+      <c r="B17" s="8" t="b">
         <v>0</v>
       </c>
       <c r="C17" s="3" t="s">
@@ -2476,100 +2508,100 @@
     </row>
     <row r="2" spans="1:25" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>69</v>
+        <v>62</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
         <v>73</v>
-      </c>
-      <c r="B4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="D4" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" t="s">
         <v>66</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="D5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="14.25" customHeight="1">
       <c r="A6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" t="s">
         <v>64</v>
-      </c>
-      <c r="B6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="D6" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:25" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>69</v>
+        <v>107</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="14.4">
-      <c r="A8" s="14" t="s">
-        <v>136</v>
+      <c r="A8" s="12" t="s">
+        <v>135</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>62</v>
+        <v>135</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>61</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1"/>
@@ -3545,71 +3577,71 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="7"/>
+    <col min="6" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="13" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="11" customFormat="1" ht="230.4">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:5" s="9" customFormat="1" ht="230.4">
+      <c r="A2" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="D2" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="E2" s="17" t="s">
+      <c r="C2" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="201.6">
+      <c r="A3" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="15" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="201.6">
-      <c r="A3" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>61</v>
-      </c>
-    </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="13"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="12"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3621,53 +3653,53 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.109375" style="7"/>
+    <col min="1" max="1" width="13.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="161.33203125" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="13" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="158.4">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:4" ht="259.2">
+      <c r="A2" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="187.2">
-      <c r="A3" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="B3" s="18" t="s">
+      <c r="C2" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="374.4">
+      <c r="A3" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>138</v>
+      <c r="C3" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated - HTML in the send email and File retention component
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://qbotica-my.sharepoint.com/personal/premkumar_sivakumar_qbotica_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="14_{2AA3EA44-538C-46F1-80C7-01D43EBC6AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F6FDDF0-CAC3-4BF4-86C7-E6DBE390082B}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="14_{2AA3EA44-538C-46F1-80C7-01D43EBC6AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B74AB44-0C3D-4126-A375-C092B3F4C1C5}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="144">
   <si>
     <t>Name</t>
   </si>
@@ -449,16 +449,10 @@
     <t>EM0002</t>
   </si>
   <si>
-    <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
-  </si>
-  <si>
     <t>BillingForecastTemplate_DSName</t>
   </si>
   <si>
     <t>BillingForecastTemplateMap</t>
-  </si>
-  <si>
-    <t>mercury@inpwrinc.com</t>
   </si>
   <si>
     <t>Billing forecast for 24114</t>
@@ -509,6 +503,9 @@
   Regards,&lt;br/&gt;
   Bot
 &lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>mercury@inpwrinc.com;calypso@inpwrinc.com;pegasus@inpwrinc.com</t>
   </si>
 </sst>
 </file>
@@ -621,10 +618,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1172,10 +1169,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>138</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -3609,8 +3606,8 @@
       <c r="B2" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="16" t="s">
-        <v>137</v>
+      <c r="C2" s="17" t="s">
+        <v>143</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>47</v>
@@ -3626,8 +3623,8 @@
       <c r="B3" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>137</v>
+      <c r="C3" s="17" t="s">
+        <v>143</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>54</v>
@@ -3678,28 +3675,28 @@
       <c r="A2" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>140</v>
+      <c r="B2" s="17" t="s">
+        <v>143</v>
       </c>
       <c r="C2" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" s="16" t="s">
         <v>141</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="374.4">
       <c r="A3" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="C3" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" s="16" t="s">
         <v>142</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated - Send email with all PDF files and current Month date asset update
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://qbotica-my.sharepoint.com/personal/premkumar_sivakumar_qbotica_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="14_{2AA3EA44-538C-46F1-80C7-01D43EBC6AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B74AB44-0C3D-4126-A375-C092B3F4C1C5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201C9ACB-CDF9-434E-8C3A-E49E02DB3D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="147">
   <si>
     <t>Name</t>
   </si>
@@ -506,6 +506,15 @@
   </si>
   <si>
     <t>mercury@inpwrinc.com;calypso@inpwrinc.com;pegasus@inpwrinc.com</t>
+  </si>
+  <si>
+    <t>CurrentMonthEndDate_AssetFolder</t>
+  </si>
+  <si>
+    <t>CurrentMonthEndDate_AssetName</t>
+  </si>
+  <si>
+    <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
   </si>
 </sst>
 </file>
@@ -574,7 +583,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -620,8 +629,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -939,16 +951,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y38"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="14.4"/>
+  <dimension ref="A1:Y41"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="46.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.44140625" customWidth="1"/>
-    <col min="4" max="25" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="67.42578125" customWidth="1"/>
+    <col min="4" max="25" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="18">
+    <row r="1" spans="1:25" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1291,6 +1303,22 @@
         <v>134</v>
       </c>
     </row>
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
+        <v>144</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" t="s">
+        <v>145</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>135</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1301,12 +1329,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" style="8" customWidth="1"/>
-    <col min="3" max="3" width="75.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col min="3" max="3" width="75.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1343,7 +1371,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="28.8">
+    <row r="2" spans="1:26" ht="30">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1354,7 +1382,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -1468,7 +1496,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="28.8">
+    <row r="17" spans="1:3" ht="45">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -2460,12 +2488,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Y969"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="32.88671875" customWidth="1"/>
-    <col min="2" max="2" width="31.109375" customWidth="1"/>
-    <col min="3" max="3" width="30.33203125" customWidth="1"/>
-    <col min="4" max="25" width="65.44140625" customWidth="1"/>
+    <col min="1" max="1" width="32.85546875" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" customWidth="1"/>
+    <col min="4" max="25" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="14.25" customHeight="1">
@@ -2587,7 +2615,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="14.4">
+    <row r="8" spans="1:25">
       <c r="A8" s="12" t="s">
         <v>135</v>
       </c>
@@ -3572,17 +3600,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A045ED-89B2-46F5-87BB-9D73B35EE197}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="5"/>
+    <col min="4" max="4" width="26.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18">
+    <row r="1" spans="1:5" ht="18.75">
       <c r="A1" s="13" t="s">
         <v>42</v>
       </c>
@@ -3599,7 +3627,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="9" customFormat="1" ht="230.4">
+    <row r="2" spans="1:5" s="9" customFormat="1" ht="240">
       <c r="A2" s="14" t="s">
         <v>43</v>
       </c>
@@ -3616,7 +3644,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="201.6">
+    <row r="3" spans="1:5" ht="210">
       <c r="A3" s="14" t="s">
         <v>53</v>
       </c>
@@ -3648,16 +3676,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7C6B43-6EA4-4DD0-939E-D4A6AD374EA2}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="161.33203125" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="13.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="161.28515625" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18">
+    <row r="1" spans="1:4" ht="18.75">
       <c r="A1" s="13" t="s">
         <v>45</v>
       </c>
@@ -3671,12 +3699,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="259.2">
+    <row r="2" spans="1:4" ht="270">
       <c r="A2" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="17" t="s">
-        <v>143</v>
+      <c r="B2" s="18" t="s">
+        <v>146</v>
       </c>
       <c r="C2" s="14" t="s">
         <v>139</v>
@@ -3685,12 +3713,12 @@
         <v>141</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="374.4">
+    <row r="3" spans="1:4" ht="390">
       <c r="A3" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="B3" s="17" t="s">
-        <v>143</v>
+      <c r="B3" s="18" t="s">
+        <v>146</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>140</v>

</xml_diff>

<commit_message>
Updated Asset Values which align with Common Utilities
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://qbotica-my.sharepoint.com/personal/premkumar_sivakumar_qbotica_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201C9ACB-CDF9-434E-8C3A-E49E02DB3D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:1_{201C9ACB-CDF9-434E-8C3A-E49E02DB3D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD939368-58DF-412F-8407-032712A52934}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="148">
   <si>
     <t>Name</t>
   </si>
@@ -242,15 +242,9 @@
     <t>Cred_Office365_AppID</t>
   </si>
   <si>
-    <t>Billing</t>
-  </si>
-  <si>
     <t>The Login URL for Spectrum</t>
   </si>
   <si>
-    <t>Spectrum_URL</t>
-  </si>
-  <si>
     <t>Cred_SpectrumLogin</t>
   </si>
   <si>
@@ -360,9 +354,6 @@
   </si>
   <si>
     <t>DataService_RefreshToken</t>
-  </si>
-  <si>
-    <t>AP_DataService_API</t>
   </si>
   <si>
     <t>Client Secret Id for the Data Service within the API scope.</t>
@@ -508,13 +499,25 @@
     <t>mercury@inpwrinc.com;calypso@inpwrinc.com;pegasus@inpwrinc.com</t>
   </si>
   <si>
-    <t>CurrentMonthEndDate_AssetFolder</t>
-  </si>
-  <si>
-    <t>CurrentMonthEndDate_AssetName</t>
-  </si>
-  <si>
     <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
+  </si>
+  <si>
+    <t>Report name</t>
+  </si>
+  <si>
+    <t>Common Utilities</t>
+  </si>
+  <si>
+    <t>SpectrumLogin_URL</t>
+  </si>
+  <si>
+    <t>O365_Application</t>
+  </si>
+  <si>
+    <t>SpectrumLogin_Account</t>
+  </si>
+  <si>
+    <t>DataService_API</t>
   </si>
 </sst>
 </file>
@@ -561,12 +564,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -583,7 +592,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -632,8 +641,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -951,16 +966,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y41"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:Y38"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.42578125" customWidth="1"/>
-    <col min="4" max="25" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="46.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="67.44140625" customWidth="1"/>
+    <col min="4" max="25" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="18.75">
+    <row r="1" spans="1:25" ht="18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -998,7 +1013,7 @@
         <v>20</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>51</v>
@@ -1006,7 +1021,7 @@
     </row>
     <row r="3" spans="1:25">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B3" s="7">
         <v>3</v>
@@ -1017,7 +1032,7 @@
     </row>
     <row r="4" spans="1:25">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B4" s="7">
         <v>30</v>
@@ -1028,7 +1043,7 @@
     </row>
     <row r="5" spans="1:25">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>50</v>
@@ -1039,46 +1054,46 @@
     </row>
     <row r="6" spans="1:25">
       <c r="A6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:25">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" t="s">
-        <v>80</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>68</v>
+        <v>78</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>143</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1086,21 +1101,21 @@
         <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>67</v>
+        <v>145</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>71</v>
+        <v>146</v>
       </c>
       <c r="C11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1113,210 +1128,203 @@
     </row>
     <row r="14" spans="1:25">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:25">
       <c r="A15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>85</v>
-      </c>
       <c r="C15" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:25">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="C17" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B18" s="8" t="s">
         <v>61</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C19" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="B26" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>110</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>68</v>
+        <v>107</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>143</v>
       </c>
       <c r="C27" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C29" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>129</v>
+        <v>126</v>
+      </c>
+      <c r="C31" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
+        <v>122</v>
+      </c>
+      <c r="B32" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="C32" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>123</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C33" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>127</v>
+      </c>
+      <c r="B35" s="8" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
-      <c r="A33" t="s">
-        <v>126</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2">
-      <c r="A35" t="s">
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>129</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
         <v>130</v>
       </c>
-      <c r="B35" s="8" t="s">
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
         <v>131</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
-      <c r="A36" t="s">
-        <v>132</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2">
-      <c r="A37" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
-      <c r="A38" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2">
-      <c r="A40" t="s">
-        <v>144</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2">
-      <c r="A41" t="s">
-        <v>145</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1329,12 +1337,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" style="8" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1371,7 +1379,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="28.8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1382,7 +1390,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -1496,7 +1504,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
+    <row r="17" spans="1:3" ht="28.8">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -2488,12 +2496,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Y969"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="32.85546875" customWidth="1"/>
-    <col min="2" max="2" width="31.140625" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="25" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="32.88671875" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" customWidth="1"/>
+    <col min="3" max="3" width="30.33203125" customWidth="1"/>
+    <col min="4" max="25" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="14.25" customHeight="1">
@@ -2539,7 +2547,7 @@
         <v>62</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>56</v>
@@ -2547,30 +2555,30 @@
     </row>
     <row r="3" spans="1:25" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>70</v>
+        <v>144</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="14.25" customHeight="1">
@@ -2603,30 +2611,30 @@
     </row>
     <row r="7" spans="1:25" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>68</v>
+        <v>105</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>143</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" ht="14.4">
       <c r="A8" s="12" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>61</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1"/>
@@ -3600,17 +3608,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A045ED-89B2-46F5-87BB-9D73B35EE197}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="5"/>
+    <col min="4" max="4" width="26.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75">
+    <row r="1" spans="1:5" ht="18">
       <c r="A1" s="13" t="s">
         <v>42</v>
       </c>
@@ -3627,7 +3635,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="9" customFormat="1" ht="240">
+    <row r="2" spans="1:5" s="9" customFormat="1" ht="230.4">
       <c r="A2" s="14" t="s">
         <v>43</v>
       </c>
@@ -3635,7 +3643,7 @@
         <v>44</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>47</v>
@@ -3644,7 +3652,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="210">
+    <row r="3" spans="1:5" ht="201.6">
       <c r="A3" s="14" t="s">
         <v>53</v>
       </c>
@@ -3652,7 +3660,7 @@
         <v>55</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>54</v>
@@ -3676,16 +3684,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7C6B43-6EA4-4DD0-939E-D4A6AD374EA2}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="161.28515625" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="13.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="161.33203125" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75">
+    <row r="1" spans="1:4" ht="18">
       <c r="A1" s="13" t="s">
         <v>45</v>
       </c>
@@ -3699,32 +3707,32 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="270">
+    <row r="2" spans="1:4" ht="259.2">
       <c r="A2" s="14" t="s">
         <v>46</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C2" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="374.4">
+      <c r="A3" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" s="16" t="s">
         <v>139</v>
-      </c>
-      <c r="D2" s="16" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="390">
-      <c r="A3" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added asset for CTSR and BHR from date selection
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D642C2EF-4C97-4E79-96BA-1AC27736A125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B42699-C361-4AE3-9083-261FB564DE32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="202">
   <si>
     <t>Name</t>
   </si>
@@ -446,12 +446,6 @@
     <t>BillingForecastTemplateMap</t>
   </si>
   <si>
-    <t>Billing forecast for 24114</t>
-  </si>
-  <si>
-    <t>Billing forecast for 24114 with BRE</t>
-  </si>
-  <si>
     <t>mercury@inpwrinc.com;calypso@inpwrinc.com;pegasus@inpwrinc.com</t>
   </si>
   <si>
@@ -587,13 +581,52 @@
     <t>ReportName</t>
   </si>
   <si>
-    <t>24114 - CACI Crane - Billing Forecast</t>
-  </si>
-  <si>
     <t>Report_SPFolderPath</t>
   </si>
   <si>
     <t>Sharepoint Folder to upload report files</t>
+  </si>
+  <si>
+    <t>BF_O365_MailAccount</t>
+  </si>
+  <si>
+    <t>Mail Id used for Bot used for Trigger</t>
+  </si>
+  <si>
+    <t>BF_O365_MailFolder_Exception</t>
+  </si>
+  <si>
+    <t>BF_O365_MailFolder_Completed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exception mail folder name </t>
+  </si>
+  <si>
+    <t>Completed mail folder name</t>
+  </si>
+  <si>
+    <t>BF_ProcessName</t>
+  </si>
+  <si>
+    <t>Billing Forecast</t>
+  </si>
+  <si>
+    <t>Inbox\Billing Forecast\Completed</t>
+  </si>
+  <si>
+    <t>Inbox\Billing Forecast\Exceptions</t>
+  </si>
+  <si>
+    <t>Process name used to get it from Subject</t>
+  </si>
+  <si>
+    <t>BF_O365_MailFolder_Inbox</t>
+  </si>
+  <si>
+    <t>Inbox\Billing Forecast\New Requests</t>
+  </si>
+  <si>
+    <t>CTSRFromDate</t>
   </si>
   <si>
     <t>&lt;style&gt;
@@ -607,7 +640,7 @@
   }
 &lt;/style&gt;
 &lt;p&gt;
-Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have processed the Billing forecast for &lt;strong&gt;24114 – CACI CRANE&lt;/strong&gt;. Attached are the spectrum reports &amp; the updated template for the Month {0}. &lt;br/&gt;We observed few verification mis-matches as below, 
+Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have processed the Billing forecast for &lt;strong&gt;{1}&lt;/strong&gt;. Attached are the spectrum reports &amp; the updated template for the Month {0}. &lt;br/&gt;We observed few verification mis-matches as below, 
 &lt;/p&gt;
 SharePoint Report Path: {Path}
 &lt;p&gt;Business Rule Excetions: &lt;/p&gt;
@@ -624,8 +657,7 @@
   </si>
   <si>
     <t>&lt;p&gt;
- Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have successfully processed the billing forecast for 
-  &lt;strong&gt;24114 – CACI CRANE&lt;/strong&gt;. Attached are the Spectrum reports 
+ Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have successfully processed the billing forecast for &lt;strong&gt;{1}&lt;/strong&gt;. Attached are the Spectrum reports 
   and the updated template for the month {0}
 &lt;/p&gt;
 SharePoint Report Path: {Path}
@@ -640,6 +672,15 @@
   Regards,&lt;br/&gt;
   Bot
 &lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>BHRFromDate</t>
+  </si>
+  <si>
+    <t>Billing Forecast Report for &lt;JOBNUM&gt;</t>
+  </si>
+  <si>
+    <t>Billing Forecast Report for &lt;JOBNUM&gt; with BRE</t>
   </si>
 </sst>
 </file>
@@ -1088,7 +1129,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y58"/>
+  <dimension ref="A1:Y63"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
@@ -1212,7 +1253,7 @@
         <v>78</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C9" t="s">
         <v>102</v>
@@ -1223,7 +1264,7 @@
         <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C10" t="s">
         <v>103</v>
@@ -1234,19 +1275,15 @@
         <v>69</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C11" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:25">
-      <c r="A12" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>183</v>
-      </c>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
     </row>
     <row r="13" spans="1:25">
       <c r="A13" s="2"/>
@@ -1363,10 +1400,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B26" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>106</v>
@@ -1377,7 +1414,7 @@
         <v>107</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C27" t="s">
         <v>102</v>
@@ -1402,7 +1439,7 @@
         <v>126</v>
       </c>
       <c r="C31" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1413,7 +1450,7 @@
         <v>125</v>
       </c>
       <c r="C32" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1424,7 +1461,7 @@
         <v>124</v>
       </c>
       <c r="C33" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1455,146 +1492,187 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
+        <v>164</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>165</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
         <v>166</v>
       </c>
-      <c r="B48" s="8" t="s">
+      <c r="B50" s="8" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
-      <c r="A49" t="s">
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
         <v>167</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B51" s="8" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
-      <c r="A50" t="s">
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
         <v>168</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="B52" s="8" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
-      <c r="A51" t="s">
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
         <v>169</v>
       </c>
-      <c r="B51" s="8" t="s">
+      <c r="B53" s="8" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
-      <c r="A52" t="s">
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
         <v>170</v>
       </c>
-      <c r="B52" s="8" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="A53" t="s">
+      <c r="B54" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="B53" s="8" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2">
-      <c r="A54" t="s">
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
         <v>172</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B55" s="8" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
-      <c r="A55" t="s">
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
         <v>174</v>
       </c>
-      <c r="B55" s="8" t="s">
+      <c r="B56" s="8" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="56" spans="1:2">
-      <c r="A56" t="s">
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
         <v>176</v>
       </c>
-      <c r="B56" s="8" t="s">
+      <c r="B57" s="8" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
-      <c r="A57" t="s">
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>179</v>
+      </c>
+      <c r="B58" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="B57" s="8" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
-      <c r="A58" t="s">
-        <v>181</v>
-      </c>
-      <c r="B58" s="8" t="s">
-        <v>180</v>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>194</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>185</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="C61" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>186</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="C62" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>189</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C63" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -2825,13 +2903,13 @@
     </row>
     <row r="3" spans="1:25" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>68</v>
@@ -2887,7 +2965,7 @@
         <v>105</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>104</v>
@@ -2909,22 +2987,65 @@
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B9" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>61</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:25" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:25" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:25" ht="14.25" customHeight="1"/>
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>183</v>
+      </c>
+      <c r="B10" t="s">
+        <v>183</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
+        <v>196</v>
+      </c>
+      <c r="B11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" ht="14.25" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" ht="14.25" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
     <row r="14" spans="1:25" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:25" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:25" ht="14.25" customHeight="1"/>
@@ -3926,7 +4047,7 @@
         <v>44</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>47</v>
@@ -3943,7 +4064,7 @@
         <v>55</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>54</v>
@@ -3972,7 +4093,7 @@
     <col min="1" max="1" width="13.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.5703125" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="161.28515625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="167.5703125" style="4" customWidth="1"/>
     <col min="5" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
@@ -3990,18 +4111,18 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="285">
+    <row r="2" spans="1:4" ht="270">
       <c r="A2" s="14" t="s">
         <v>46</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>136</v>
+        <v>200</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="409.5">
@@ -4009,13 +4130,13 @@
         <v>133</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>137</v>
+        <v>201</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated with new Billing Forecast template and new vendor types
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B42699-C361-4AE3-9083-261FB564DE32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A49957-341A-43E6-BE01-C2EF2BC415E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -19,12 +19,25 @@
     <sheet name="Exceptions" sheetId="4" r:id="rId4"/>
     <sheet name="Emails" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="213">
   <si>
     <t>Name</t>
   </si>
@@ -305,9 +318,6 @@
     <t>BillingForecastTemplate_AssetFolder</t>
   </si>
   <si>
-    <t>24114_BillingForecast.xlsx</t>
-  </si>
-  <si>
     <t>BillingForecastTemplate_Name</t>
   </si>
   <si>
@@ -428,12 +438,6 @@
     <t>BHR_Division</t>
   </si>
   <si>
-    <t>BHR_From_GL_Date</t>
-  </si>
-  <si>
-    <t>BHR_From_Invoice_Date</t>
-  </si>
-  <si>
     <t>CurrentMonth_EndDate</t>
   </si>
   <si>
@@ -446,15 +450,9 @@
     <t>BillingForecastTemplateMap</t>
   </si>
   <si>
-    <t>mercury@inpwrinc.com;calypso@inpwrinc.com;pegasus@inpwrinc.com</t>
-  </si>
-  <si>
     <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
   </si>
   <si>
-    <t>Report name</t>
-  </si>
-  <si>
     <t>Common Utilities</t>
   </si>
   <si>
@@ -551,28 +549,13 @@
     <t>JOR_ContractAmount</t>
   </si>
   <si>
-    <t>C14</t>
-  </si>
-  <si>
     <t>JOR_GrossProfit</t>
   </si>
   <si>
-    <t>C15</t>
-  </si>
-  <si>
     <t>JOR_GrossPercenrtage</t>
   </si>
   <si>
-    <t>D15</t>
-  </si>
-  <si>
     <t>JOR_BillingForeCastAmount</t>
-  </si>
-  <si>
-    <t>C18</t>
-  </si>
-  <si>
-    <t>B21</t>
   </si>
   <si>
     <t>JOR_CompletionDate</t>
@@ -681,6 +664,69 @@
   </si>
   <si>
     <t>Billing Forecast Report for &lt;JOBNUM&gt; with BRE</t>
+  </si>
+  <si>
+    <t>JOR_Burden_Projection</t>
+  </si>
+  <si>
+    <t>JOR_Fringe_Projection</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>C17</t>
+  </si>
+  <si>
+    <t>D17</t>
+  </si>
+  <si>
+    <t>C20</t>
+  </si>
+  <si>
+    <t>B23</t>
+  </si>
+  <si>
+    <t>CTSR_BurdenTotal</t>
+  </si>
+  <si>
+    <t>CTSR_FringeTotal</t>
+  </si>
+  <si>
+    <t>Z10</t>
+  </si>
+  <si>
+    <t>Z11</t>
+  </si>
+  <si>
+    <t>Report name of JOR</t>
+  </si>
+  <si>
+    <t>Report name of CTSR</t>
+  </si>
+  <si>
+    <t>Report name of BHR</t>
+  </si>
+  <si>
+    <t>Billing Forecast Template.xlsx</t>
+  </si>
+  <si>
+    <t>mercury@inpwrinc.com;calypso@inpwrinc.com;</t>
+  </si>
+  <si>
+    <t>BHR_BillingForecastAmount</t>
+  </si>
+  <si>
+    <t>BHR_BHRTotalAmount</t>
+  </si>
+  <si>
+    <t>Z20</t>
   </si>
 </sst>
 </file>
@@ -802,9 +848,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -812,6 +855,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1129,7 +1175,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y63"/>
+  <dimension ref="A1:Y70"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
@@ -1176,7 +1222,7 @@
         <v>20</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>51</v>
@@ -1220,10 +1266,10 @@
         <v>75</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" t="s">
         <v>94</v>
-      </c>
-      <c r="C6" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1234,7 +1280,7 @@
         <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1245,18 +1291,18 @@
         <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="20" t="s">
-        <v>139</v>
+      <c r="B9" s="19" t="s">
+        <v>134</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1264,10 +1310,10 @@
         <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -1275,10 +1321,10 @@
         <v>69</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1324,7 +1370,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="C17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1335,344 +1381,382 @@
         <v>61</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>92</v>
-      </c>
       <c r="C19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>89</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>109</v>
-      </c>
       <c r="C25" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B26" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>107</v>
-      </c>
-      <c r="B27" s="19" t="s">
-        <v>139</v>
+        <v>106</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>134</v>
       </c>
       <c r="C27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
+        <v>111</v>
+      </c>
+      <c r="B29" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="C29" t="s">
         <v>113</v>
-      </c>
-      <c r="C29" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C31" t="s">
-        <v>138</v>
+        <v>205</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C32" t="s">
-        <v>138</v>
+        <v>206</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
+        <v>122</v>
+      </c>
+      <c r="B33" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="B33" s="8" t="s">
-        <v>124</v>
-      </c>
       <c r="C33" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
+        <v>126</v>
+      </c>
+      <c r="B35" s="8" t="s">
         <v>127</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>131</v>
+        <v>139</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>145</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>153</v>
+        <v>201</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>149</v>
+        <v>203</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
+        <v>159</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>160</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>161</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
+        <v>162</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" t="s">
+        <v>163</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
+        <v>192</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
+        <v>193</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
         <v>164</v>
       </c>
-      <c r="B48" s="8" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" t="s">
+      <c r="B55" s="8" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
         <v>165</v>
       </c>
-      <c r="B49" s="8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="A50" t="s">
+      <c r="B56" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
         <v>166</v>
       </c>
-      <c r="B50" s="8" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3">
-      <c r="A51" t="s">
+      <c r="B57" s="8" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
         <v>167</v>
       </c>
-      <c r="B51" s="8" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" t="s">
+      <c r="B58" s="8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
         <v>168</v>
       </c>
-      <c r="B52" s="8" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" t="s">
+      <c r="B59" s="8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
         <v>169</v>
       </c>
-      <c r="B53" s="8" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54" t="s">
-        <v>170</v>
-      </c>
-      <c r="B54" s="8" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" t="s">
-        <v>172</v>
-      </c>
-      <c r="B55" s="8" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="A56" t="s">
-        <v>174</v>
-      </c>
-      <c r="B56" s="8" t="s">
+      <c r="B60" s="8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" t="s">
+        <v>210</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" t="s">
+        <v>211</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>184</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="A57" t="s">
+      <c r="B68" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C68" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
         <v>176</v>
       </c>
-      <c r="B57" s="8" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58" t="s">
+      <c r="B69" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="C69" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
         <v>179</v>
       </c>
-      <c r="B58" s="8" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3">
-      <c r="A60" t="s">
-        <v>194</v>
-      </c>
-      <c r="B60" s="8" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3">
-      <c r="A61" t="s">
-        <v>185</v>
-      </c>
-      <c r="B61" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="C61" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3">
-      <c r="A62" t="s">
-        <v>186</v>
-      </c>
-      <c r="B62" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="C62" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63" t="s">
-        <v>189</v>
-      </c>
-      <c r="B63" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="C63" t="s">
-        <v>193</v>
+      <c r="B70" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="C70" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -2903,13 +2987,13 @@
     </row>
     <row r="3" spans="1:25" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>139</v>
+        <v>135</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>134</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>68</v>
@@ -2959,66 +3043,66 @@
     </row>
     <row r="7" spans="1:25" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>139</v>
+        <v>104</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>134</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" s="12" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>61</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="B9" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>61</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="B10" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>61</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="14.25" customHeight="1">
       <c r="A11" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="B11" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>61</v>
@@ -3026,10 +3110,10 @@
     </row>
     <row r="12" spans="1:25" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>61</v>
@@ -3037,10 +3121,10 @@
     </row>
     <row r="13" spans="1:25" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>61</v>
@@ -4016,7 +4100,7 @@
   <cols>
     <col min="1" max="1" width="18.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" style="5" customWidth="1"/>
     <col min="4" max="4" width="26.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="5"/>
@@ -4046,8 +4130,8 @@
       <c r="B2" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="17" t="s">
-        <v>136</v>
+      <c r="C2" s="20" t="s">
+        <v>209</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>47</v>
@@ -4063,8 +4147,8 @@
       <c r="B3" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="17" t="s">
-        <v>136</v>
+      <c r="C3" s="20" t="s">
+        <v>209</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>54</v>
@@ -4115,28 +4199,28 @@
       <c r="A2" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>137</v>
+      <c r="B2" s="17" t="s">
+        <v>133</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="409.5">
       <c r="A3" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="B3" s="18" t="s">
-        <v>137</v>
-      </c>
       <c r="C3" s="14" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Billing Forecast - Major Code change for Dynamic report preparation for Billing Forecast Template and data population,
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A49957-341A-43E6-BE01-C2EF2BC415E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C1BDE7-EC24-4A4D-90EB-F36D5F8BB90D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="225">
   <si>
     <t>Name</t>
   </si>
@@ -234,9 +234,6 @@
 Support Team</t>
   </si>
   <si>
-    <t>Billing/24114 Billing Forecast</t>
-  </si>
-  <si>
     <t>Spectrum_Environment_Code</t>
   </si>
   <si>
@@ -246,12 +243,6 @@
     <t>mail Id used for reading/ sending the bot process emails</t>
   </si>
   <si>
-    <t>Job_Number</t>
-  </si>
-  <si>
-    <t>The job number for which forecasting is done</t>
-  </si>
-  <si>
     <t>Cred_Office365_AppID</t>
   </si>
   <si>
@@ -466,42 +457,6 @@
   </si>
   <si>
     <t>DataService_API</t>
-  </si>
-  <si>
-    <t>CTSR_EquipmentTotal</t>
-  </si>
-  <si>
-    <t>Z4</t>
-  </si>
-  <si>
-    <t>Z5</t>
-  </si>
-  <si>
-    <t>Z6</t>
-  </si>
-  <si>
-    <t>Z7</t>
-  </si>
-  <si>
-    <t>Z8</t>
-  </si>
-  <si>
-    <t>CTSR_LaborTotal</t>
-  </si>
-  <si>
-    <t>CTSR_MaterialTotal</t>
-  </si>
-  <si>
-    <t>CTSR_OthersTotal</t>
-  </si>
-  <si>
-    <t>CTSR_SubsTotal</t>
-  </si>
-  <si>
-    <t>CTSR_TravellTotal</t>
-  </si>
-  <si>
-    <t>Z9</t>
   </si>
   <si>
     <t>JOR_Equipment_Projection</t>
@@ -693,18 +648,6 @@
     <t>B23</t>
   </si>
   <si>
-    <t>CTSR_BurdenTotal</t>
-  </si>
-  <si>
-    <t>CTSR_FringeTotal</t>
-  </si>
-  <si>
-    <t>Z10</t>
-  </si>
-  <si>
-    <t>Z11</t>
-  </si>
-  <si>
     <t>Report name of JOR</t>
   </si>
   <si>
@@ -727,13 +670,106 @@
   </si>
   <si>
     <t>Z20</t>
+  </si>
+  <si>
+    <t>BillingForecast_QueueFolder</t>
+  </si>
+  <si>
+    <t>BillingForecast_QueueName</t>
+  </si>
+  <si>
+    <t>BillingForecast_JobQueue</t>
+  </si>
+  <si>
+    <t>Local_ReportsFolder_AssetFolder</t>
+  </si>
+  <si>
+    <t>Local_ReportsFolder_Name</t>
+  </si>
+  <si>
+    <t>JobReportName</t>
+  </si>
+  <si>
+    <t>&amp;=SUM(C4:C11)</t>
+  </si>
+  <si>
+    <t>JOR_GrossProfit_Formula</t>
+  </si>
+  <si>
+    <t>&amp;=C16-C12</t>
+  </si>
+  <si>
+    <t>JOR_Total_Projection_Formula</t>
+  </si>
+  <si>
+    <t>Equip_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>D8</t>
+  </si>
+  <si>
+    <t>D9</t>
+  </si>
+  <si>
+    <t>D10</t>
+  </si>
+  <si>
+    <t>D11</t>
+  </si>
+  <si>
+    <t>D12</t>
+  </si>
+  <si>
+    <t>Labor_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Material_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Others_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Subs_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Travel_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Burden_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Fringe_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Total_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Profit_AmountToAllocate_Formula</t>
+  </si>
+  <si>
+    <t>&amp;=C17/C16</t>
+  </si>
+  <si>
+    <t>Billing/Billing Forecast</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -772,6 +808,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -801,7 +843,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -858,6 +900,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1175,7 +1221,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y70"/>
+  <dimension ref="A1:Y82"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
@@ -1222,7 +1268,7 @@
         <v>20</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>51</v>
@@ -1230,7 +1276,7 @@
     </row>
     <row r="3" spans="1:25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B3" s="7">
         <v>3</v>
@@ -1241,7 +1287,7 @@
     </row>
     <row r="4" spans="1:25">
       <c r="A4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B4" s="7">
         <v>30</v>
@@ -1252,7 +1298,7 @@
     </row>
     <row r="5" spans="1:25">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>50</v>
@@ -1263,68 +1309,68 @@
     </row>
     <row r="6" spans="1:25">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:25">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:25">
       <c r="A10" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C10" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C11" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1337,426 +1383,500 @@
     </row>
     <row r="14" spans="1:25">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:25">
       <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" t="s">
         <v>81</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:25">
       <c r="A16" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C16" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="C17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" t="s">
+      <c r="A18" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>224</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="B19" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>90</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" t="s">
-        <v>98</v>
+      <c r="C19" s="21" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" t="s">
-        <v>89</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>208</v>
-      </c>
+      <c r="A20" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C20" s="21"/>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" t="s">
-        <v>131</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>132</v>
-      </c>
+      <c r="A21" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21" s="21"/>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B26" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C29" t="s">
-        <v>113</v>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>198</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>120</v>
+        <v>197</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="C31" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>121</v>
+        <v>199</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="C32" t="s">
-        <v>206</v>
+        <v>155</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="B33" s="8" t="s">
-        <v>123</v>
-      </c>
       <c r="C33" t="s">
-        <v>207</v>
+        <v>186</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="C34" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>128</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>127</v>
+        <v>120</v>
+      </c>
+      <c r="C35" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>123</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>145</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>146</v>
+        <v>204</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>142</v>
+        <v>205</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>147</v>
+        <v>214</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>143</v>
+        <v>206</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>148</v>
+        <v>215</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>144</v>
+        <v>207</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>149</v>
+        <v>216</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>150</v>
+        <v>208</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>204</v>
+        <v>210</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>219</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>151</v>
+        <v>220</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>152</v>
+        <v>212</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>159</v>
+        <v>221</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>153</v>
+        <v>213</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>160</v>
+        <v>222</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2">
-      <c r="A50" t="s">
-        <v>161</v>
-      </c>
-      <c r="B50" s="8" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2">
-      <c r="A51" t="s">
-        <v>162</v>
-      </c>
-      <c r="B51" s="8" t="s">
-        <v>156</v>
+        <v>223</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
-        <v>163</v>
+        <v>136</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
-        <v>192</v>
+        <v>144</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>158</v>
+        <v>138</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" t="s">
-        <v>193</v>
+        <v>145</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>194</v>
+        <v>139</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>195</v>
+        <v>140</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>196</v>
+        <v>141</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>197</v>
+        <v>142</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>198</v>
+        <v>143</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>199</v>
+        <v>179</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" t="s">
-        <v>169</v>
+        <v>149</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>200</v>
+        <v>180</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" t="s">
+        <v>150</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" t="s">
-        <v>210</v>
+        <v>151</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" t="s">
-        <v>211</v>
+        <v>152</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>212</v>
+        <v>183</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" t="s">
+        <v>153</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>154</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>203</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>184</v>
+        <v>201</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3">
-      <c r="A68" t="s">
-        <v>175</v>
-      </c>
-      <c r="B68" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="C68" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3">
-      <c r="A69" t="s">
-        <v>176</v>
-      </c>
-      <c r="B69" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="C69" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="C70" t="s">
-        <v>183</v>
+        <v>184</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>192</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
+        <v>169</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" t="s">
+        <v>160</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="C76" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" t="s">
+        <v>161</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C77" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" t="s">
+        <v>164</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C78" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
+        <v>194</v>
+      </c>
+      <c r="B81" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
+        <v>195</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -2973,13 +3093,13 @@
     </row>
     <row r="2" spans="1:25" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>61</v>
+        <v>224</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>56</v>
@@ -2987,147 +3107,138 @@
     </row>
     <row r="3" spans="1:25" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>61</v>
+        <v>224</v>
       </c>
       <c r="D4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="14.25" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D5" t="s">
-        <v>66</v>
-      </c>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="7"/>
     </row>
     <row r="6" spans="1:25" ht="14.25" customHeight="1">
       <c r="A6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D6" t="s">
         <v>63</v>
-      </c>
-      <c r="B6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D6" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:25" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" s="12" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>61</v>
+        <v>224</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="B9" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>61</v>
+        <v>224</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="B10" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>61</v>
+        <v>224</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="14.25" customHeight="1">
       <c r="A11" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="B11" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>61</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:25" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>61</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>61</v>
+        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:25" ht="14.25" customHeight="1"/>
@@ -4131,7 +4242,7 @@
         <v>44</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>209</v>
+        <v>190</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>47</v>
@@ -4148,7 +4259,7 @@
         <v>55</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>209</v>
+        <v>190</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>54</v>
@@ -4200,27 +4311,27 @@
         <v>46</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="409.5">
       <c r="A3" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="17" t="s">
-        <v>133</v>
-      </c>
       <c r="C3" s="14" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Billing Forecast - Updated Billing Forecast workflow and removed few workflows
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C1BDE7-EC24-4A4D-90EB-F36D5F8BB90D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A5273BF-4A22-4E58-988E-663DB18AA468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="215">
   <si>
     <t>Name</t>
   </si>
@@ -306,18 +306,6 @@
     <t>Billing History</t>
   </si>
   <si>
-    <t>BillingForecastTemplate_AssetFolder</t>
-  </si>
-  <si>
-    <t>BillingForecastTemplate_Name</t>
-  </si>
-  <si>
-    <t>BillingForecastTemplate_BucketName</t>
-  </si>
-  <si>
-    <t>Billing Forecast Template</t>
-  </si>
-  <si>
     <t>InPwr.Bill.BillingForecast</t>
   </si>
   <si>
@@ -333,15 +321,6 @@
     <t>Spectrum Login username and password</t>
   </si>
   <si>
-    <t>Bucket Name for Billing Forecast Report to download</t>
-  </si>
-  <si>
-    <t>Billing Forecast Report name to download</t>
-  </si>
-  <si>
-    <t>Orchestrator asset folder name for Billing to access Bucket</t>
-  </si>
-  <si>
     <t>Spectrum Login MFA code to retrieve during login process</t>
   </si>
   <si>
@@ -435,12 +414,6 @@
     <t>EM0002</t>
   </si>
   <si>
-    <t>BillingForecastTemplate_DSName</t>
-  </si>
-  <si>
-    <t>BillingForecastTemplateMap</t>
-  </si>
-  <si>
     <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
   </si>
   <si>
@@ -564,7 +537,175 @@
     <t>Inbox\Billing Forecast\New Requests</t>
   </si>
   <si>
-    <t>CTSRFromDate</t>
+    <t>Billing Forecast Report for &lt;JOBNUM&gt;</t>
+  </si>
+  <si>
+    <t>Billing Forecast Report for &lt;JOBNUM&gt; with BRE</t>
+  </si>
+  <si>
+    <t>JOR_Burden_Projection</t>
+  </si>
+  <si>
+    <t>JOR_Fringe_Projection</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>C17</t>
+  </si>
+  <si>
+    <t>D17</t>
+  </si>
+  <si>
+    <t>C20</t>
+  </si>
+  <si>
+    <t>B23</t>
+  </si>
+  <si>
+    <t>Report name of JOR</t>
+  </si>
+  <si>
+    <t>Report name of CTSR</t>
+  </si>
+  <si>
+    <t>Report name of BHR</t>
+  </si>
+  <si>
+    <t>mercury@inpwrinc.com;calypso@inpwrinc.com;</t>
+  </si>
+  <si>
+    <t>BHR_BillingForecastAmount</t>
+  </si>
+  <si>
+    <t>BHR_BHRTotalAmount</t>
+  </si>
+  <si>
+    <t>Z20</t>
+  </si>
+  <si>
+    <t>BillingForecast_QueueFolder</t>
+  </si>
+  <si>
+    <t>BillingForecast_QueueName</t>
+  </si>
+  <si>
+    <t>Local_ReportsFolder_AssetFolder</t>
+  </si>
+  <si>
+    <t>Local_ReportsFolder_Name</t>
+  </si>
+  <si>
+    <t>JobReportName</t>
+  </si>
+  <si>
+    <t>&amp;=SUM(C4:C11)</t>
+  </si>
+  <si>
+    <t>JOR_GrossProfit_Formula</t>
+  </si>
+  <si>
+    <t>&amp;=C16-C12</t>
+  </si>
+  <si>
+    <t>JOR_Total_Projection_Formula</t>
+  </si>
+  <si>
+    <t>Equip_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>D8</t>
+  </si>
+  <si>
+    <t>D9</t>
+  </si>
+  <si>
+    <t>D10</t>
+  </si>
+  <si>
+    <t>D11</t>
+  </si>
+  <si>
+    <t>D12</t>
+  </si>
+  <si>
+    <t>Labor_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Material_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Others_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Subs_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Travel_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Burden_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Fringe_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Total_AmountToAllocate</t>
+  </si>
+  <si>
+    <t>Profit_AmountToAllocate_Formula</t>
+  </si>
+  <si>
+    <t>&amp;=C17/C16</t>
+  </si>
+  <si>
+    <t>Billing/Billing Forecast</t>
+  </si>
+  <si>
+    <t>BillingForecast_JobQueue_Test</t>
+  </si>
+  <si>
+    <t>The Drive Local Folder to save reports Orchestrator Folder Name</t>
+  </si>
+  <si>
+    <t>Billing Forecast Report Name</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;
+ Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have successfully processed the billing forecast for &lt;strong&gt;{1}&lt;/strong&gt;. Attached are the Spectrum reports 
+  and the updated template for the month &lt;strong&gt;{0}&lt;/strong&gt;
+&lt;/p&gt;
+SharePoint Report Path: {Path}
+&lt;p&gt;
+  Please reach out to 
+  &lt;a href="mailto:automationsupport@inpwrinc.com"&gt;
+    automationsupport@inpwrinc.com
+  &lt;/a&gt; 
+  for any queries or clarifications.
+&lt;/p&gt;
+&lt;p&gt;
+  Regards,&lt;br/&gt;
+  Bot
+&lt;/p&gt;</t>
   </si>
   <si>
     <t>&lt;style&gt;
@@ -578,7 +719,7 @@
   }
 &lt;/style&gt;
 &lt;p&gt;
-Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have processed the Billing forecast for &lt;strong&gt;{1}&lt;/strong&gt;. Attached are the spectrum reports &amp; the updated template for the Month {0}. &lt;br/&gt;We observed few verification mis-matches as below, 
+Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have processed the Billing forecast for &lt;strong&gt;{1}&lt;/strong&gt;. Attached are the spectrum reports &amp; the updated template for the Month &lt;strong&gt;{0}&lt;/strong&gt;. &lt;br/&gt;We observed few verification mis-matches as below, 
 &lt;/p&gt;
 SharePoint Report Path: {Path}
 &lt;p&gt;Business Rule Excetions: &lt;/p&gt;
@@ -593,183 +734,12 @@
   Bot
 &lt;/p&gt;</t>
   </si>
-  <si>
-    <t>&lt;p&gt;
- Dear Automation Team,&lt;br/&gt;&lt;br/&gt; We have successfully processed the billing forecast for &lt;strong&gt;{1}&lt;/strong&gt;. Attached are the Spectrum reports 
-  and the updated template for the month {0}
-&lt;/p&gt;
-SharePoint Report Path: {Path}
-&lt;p&gt;
-  Please reach out to 
-  &lt;a href="mailto:automationsupport@inpwrinc.com"&gt;
-    automationsupport@inpwrinc.com
-  &lt;/a&gt; 
-  for any queries or clarifications.
-&lt;/p&gt;
-&lt;p&gt;
-  Regards,&lt;br/&gt;
-  Bot
-&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>BHRFromDate</t>
-  </si>
-  <si>
-    <t>Billing Forecast Report for &lt;JOBNUM&gt;</t>
-  </si>
-  <si>
-    <t>Billing Forecast Report for &lt;JOBNUM&gt; with BRE</t>
-  </si>
-  <si>
-    <t>JOR_Burden_Projection</t>
-  </si>
-  <si>
-    <t>JOR_Fringe_Projection</t>
-  </si>
-  <si>
-    <t>C11</t>
-  </si>
-  <si>
-    <t>C12</t>
-  </si>
-  <si>
-    <t>C16</t>
-  </si>
-  <si>
-    <t>C17</t>
-  </si>
-  <si>
-    <t>D17</t>
-  </si>
-  <si>
-    <t>C20</t>
-  </si>
-  <si>
-    <t>B23</t>
-  </si>
-  <si>
-    <t>Report name of JOR</t>
-  </si>
-  <si>
-    <t>Report name of CTSR</t>
-  </si>
-  <si>
-    <t>Report name of BHR</t>
-  </si>
-  <si>
-    <t>Billing Forecast Template.xlsx</t>
-  </si>
-  <si>
-    <t>mercury@inpwrinc.com;calypso@inpwrinc.com;</t>
-  </si>
-  <si>
-    <t>BHR_BillingForecastAmount</t>
-  </si>
-  <si>
-    <t>BHR_BHRTotalAmount</t>
-  </si>
-  <si>
-    <t>Z20</t>
-  </si>
-  <si>
-    <t>BillingForecast_QueueFolder</t>
-  </si>
-  <si>
-    <t>BillingForecast_QueueName</t>
-  </si>
-  <si>
-    <t>BillingForecast_JobQueue</t>
-  </si>
-  <si>
-    <t>Local_ReportsFolder_AssetFolder</t>
-  </si>
-  <si>
-    <t>Local_ReportsFolder_Name</t>
-  </si>
-  <si>
-    <t>JobReportName</t>
-  </si>
-  <si>
-    <t>&amp;=SUM(C4:C11)</t>
-  </si>
-  <si>
-    <t>JOR_GrossProfit_Formula</t>
-  </si>
-  <si>
-    <t>&amp;=C16-C12</t>
-  </si>
-  <si>
-    <t>JOR_Total_Projection_Formula</t>
-  </si>
-  <si>
-    <t>Equip_AmountToAllocate</t>
-  </si>
-  <si>
-    <t>D4</t>
-  </si>
-  <si>
-    <t>D5</t>
-  </si>
-  <si>
-    <t>D6</t>
-  </si>
-  <si>
-    <t>D7</t>
-  </si>
-  <si>
-    <t>D8</t>
-  </si>
-  <si>
-    <t>D9</t>
-  </si>
-  <si>
-    <t>D10</t>
-  </si>
-  <si>
-    <t>D11</t>
-  </si>
-  <si>
-    <t>D12</t>
-  </si>
-  <si>
-    <t>Labor_AmountToAllocate</t>
-  </si>
-  <si>
-    <t>Material_AmountToAllocate</t>
-  </si>
-  <si>
-    <t>Others_AmountToAllocate</t>
-  </si>
-  <si>
-    <t>Subs_AmountToAllocate</t>
-  </si>
-  <si>
-    <t>Travel_AmountToAllocate</t>
-  </si>
-  <si>
-    <t>Burden_AmountToAllocate</t>
-  </si>
-  <si>
-    <t>Fringe_AmountToAllocate</t>
-  </si>
-  <si>
-    <t>Total_AmountToAllocate</t>
-  </si>
-  <si>
-    <t>Profit_AmountToAllocate_Formula</t>
-  </si>
-  <si>
-    <t>&amp;=C17/C16</t>
-  </si>
-  <si>
-    <t>Billing/Billing Forecast</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -808,12 +778,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -843,7 +807,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -900,10 +864,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1221,7 +1181,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y82"/>
+  <dimension ref="A1:Y69"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
@@ -1268,7 +1228,7 @@
         <v>20</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>51</v>
@@ -1312,10 +1272,10 @@
         <v>72</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1326,7 +1286,7 @@
         <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1337,7 +1297,7 @@
         <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -1345,10 +1305,10 @@
         <v>75</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C9" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1356,10 +1316,10 @@
         <v>64</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C10" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -1367,178 +1327,199 @@
         <v>66</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
+      <c r="A12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="13" spans="1:25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="14" spans="1:25">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="C14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:25">
-      <c r="A15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C15" t="s">
-        <v>81</v>
+      <c r="A15" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:25">
-      <c r="A16" t="s">
-        <v>79</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C16" t="s">
-        <v>83</v>
+      <c r="A16" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="C17" t="s">
+      <c r="A17" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>126</v>
+      </c>
+      <c r="B18" t="s">
+        <v>126</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="B18" s="22" t="s">
-        <v>224</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>95</v>
+      <c r="B19" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>189</v>
-      </c>
-      <c r="C20" s="21"/>
+      <c r="A20" t="s">
+        <v>101</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" s="21" t="s">
-        <v>128</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="C21" s="21"/>
+      <c r="A21" t="s">
+        <v>183</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>182</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="C22" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="23" spans="1:3">
-      <c r="A23" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="A23" t="s">
+        <v>184</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C23" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="2" t="s">
+      <c r="C24" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>107</v>
+      <c r="C25" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>135</v>
-      </c>
-      <c r="B26" t="s">
-        <v>135</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
-        <v>103</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="C27" t="s">
-        <v>98</v>
+        <v>112</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C26" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>116</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="C29" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>198</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>224</v>
+        <v>190</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1546,337 +1527,272 @@
         <v>199</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>117</v>
+        <v>200</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C33" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>201</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>202</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>203</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>204</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
+        <v>205</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" t="s">
+        <v>206</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
+        <v>207</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" t="s">
+        <v>127</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>135</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
+        <v>136</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" t="s">
+        <v>137</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" t="s">
+        <v>138</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" t="s">
+        <v>139</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>164</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>165</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
+        <v>140</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
+        <v>141</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>142</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>143</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>144</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
+        <v>145</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
+        <v>188</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>118</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="B58" s="8" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
-      <c r="A35" t="s">
-        <v>119</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="C35" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>123</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" t="s">
-        <v>125</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" t="s">
-        <v>204</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" t="s">
-        <v>214</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" t="s">
-        <v>215</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" t="s">
-        <v>216</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>217</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" t="s">
-        <v>218</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" t="s">
-        <v>219</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" t="s">
-        <v>220</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48" t="s">
-        <v>221</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2">
-      <c r="A49" t="s">
-        <v>222</v>
-      </c>
-      <c r="B49" s="8" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2">
-      <c r="A52" t="s">
-        <v>136</v>
-      </c>
-      <c r="B52" s="8" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="A53" t="s">
-        <v>144</v>
-      </c>
-      <c r="B53" s="8" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2">
-      <c r="A54" t="s">
-        <v>145</v>
-      </c>
-      <c r="B54" s="8" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2">
-      <c r="A55" t="s">
-        <v>146</v>
-      </c>
-      <c r="B55" s="8" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2">
-      <c r="A56" t="s">
-        <v>147</v>
-      </c>
-      <c r="B56" s="8" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2">
-      <c r="A57" t="s">
-        <v>148</v>
-      </c>
-      <c r="B57" s="8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
-      <c r="A58" t="s">
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
         <v>177</v>
       </c>
-      <c r="B58" s="8" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2">
-      <c r="A59" t="s">
+      <c r="B60" s="8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
         <v>178</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B61" s="8" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="60" spans="1:2">
-      <c r="A60" t="s">
-        <v>149</v>
-      </c>
-      <c r="B60" s="8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2">
-      <c r="A61" t="s">
-        <v>150</v>
-      </c>
-      <c r="B61" s="8" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2">
-      <c r="A62" t="s">
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>160</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
         <v>151</v>
       </c>
-      <c r="B62" s="8" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2">
-      <c r="A63" t="s">
-        <v>152</v>
-      </c>
-      <c r="B63" s="8" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2">
-      <c r="A64" t="s">
+      <c r="B64" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C64" t="s">
         <v>153</v>
-      </c>
-      <c r="B64" s="8" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
+        <v>152</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="C65" t="s">
         <v>154</v>
-      </c>
-      <c r="B65" s="8" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>203</v>
+        <v>155</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3">
-      <c r="A67" t="s">
-        <v>201</v>
-      </c>
-      <c r="B67" s="8" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3">
-      <c r="A70" t="s">
-        <v>191</v>
-      </c>
-      <c r="B70" s="8" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3">
-      <c r="A71" t="s">
-        <v>192</v>
-      </c>
-      <c r="B71" s="8" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3">
-      <c r="A75" t="s">
-        <v>169</v>
-      </c>
-      <c r="B75" s="8" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3">
-      <c r="A76" t="s">
-        <v>160</v>
-      </c>
-      <c r="B76" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="C76" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3">
-      <c r="A77" t="s">
-        <v>161</v>
-      </c>
-      <c r="B77" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="C77" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3">
-      <c r="A78" t="s">
-        <v>164</v>
-      </c>
-      <c r="B78" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="C78" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2">
-      <c r="A81" t="s">
-        <v>194</v>
-      </c>
-      <c r="B81" s="7" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2">
-      <c r="A82" t="s">
-        <v>195</v>
-      </c>
-      <c r="B82" s="8" t="s">
-        <v>196</v>
+        <v>156</v>
+      </c>
+      <c r="C66" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
+        <v>180</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>181</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -3047,7 +2963,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Y969"/>
+  <dimension ref="A1:Y966"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="32.85546875" customWidth="1"/>
@@ -3099,7 +3015,7 @@
         <v>61</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>56</v>
@@ -3107,13 +3023,13 @@
     </row>
     <row r="3" spans="1:25" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>65</v>
@@ -3127,120 +3043,99 @@
         <v>67</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="D4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="14.25" customHeight="1">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="7"/>
+      <c r="A5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="D5" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="6" spans="1:25" ht="14.25" customHeight="1">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="D6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25">
-      <c r="A8" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>126</v>
+        <v>94</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25">
+      <c r="A7" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B8" t="s">
+        <v>147</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>111</v>
+        <v>209</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="B9" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" t="s">
-        <v>158</v>
+      <c r="A10" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>146</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25" ht="14.25" customHeight="1">
-      <c r="A11" t="s">
-        <v>171</v>
-      </c>
-      <c r="B11" t="s">
-        <v>171</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" ht="14.25" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" ht="14.25" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>224</v>
-      </c>
-    </row>
+        <v>209</v>
+      </c>
+      <c r="D10" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" ht="14.25" customHeight="1"/>
+    <row r="12" spans="1:25" ht="14.25" customHeight="1"/>
+    <row r="13" spans="1:25" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:25" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:25" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:25" ht="14.25" customHeight="1"/>
@@ -4194,9 +4089,6 @@
     <row r="964" ht="14.25" customHeight="1"/>
     <row r="965" ht="14.25" customHeight="1"/>
     <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4242,7 +4134,7 @@
         <v>44</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>47</v>
@@ -4259,7 +4151,7 @@
         <v>55</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>54</v>
@@ -4311,27 +4203,27 @@
         <v>46</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>173</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="409.5">
       <c r="A3" s="14" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>172</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Code with new formulas
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A5273BF-4A22-4E58-988E-663DB18AA468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46BFAB5C-82AF-403E-8664-DACB501D56BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="219">
   <si>
     <t>Name</t>
   </si>
@@ -679,9 +679,6 @@
   </si>
   <si>
     <t>Billing/Billing Forecast</t>
-  </si>
-  <si>
-    <t>BillingForecast_JobQueue_Test</t>
   </si>
   <si>
     <t>The Drive Local Folder to save reports Orchestrator Folder Name</t>
@@ -733,6 +730,21 @@
   Regards,&lt;br/&gt;
   Bot
 &lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>BillingForecast_JobQueue</t>
+  </si>
+  <si>
+    <t>Percent Complete</t>
+  </si>
+  <si>
+    <t>&amp;=C12/C16</t>
+  </si>
+  <si>
+    <t>Percent Complete_Forumula</t>
+  </si>
+  <si>
+    <t>C14</t>
   </si>
 </sst>
 </file>
@@ -1451,7 +1463,7 @@
         <v>209</v>
       </c>
       <c r="C22" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1462,7 +1474,7 @@
         <v>146</v>
       </c>
       <c r="C23" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1587,11 +1599,27 @@
       </c>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" t="s">
+      <c r="A40" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="7" t="s">
         <v>208</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -1792,7 +1820,7 @@
         <v>181</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -3130,7 +3158,7 @@
         <v>209</v>
       </c>
       <c r="D10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="14.25" customHeight="1"/>
@@ -4209,7 +4237,7 @@
         <v>162</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="409.5">
@@ -4223,7 +4251,7 @@
         <v>163</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Trimble upgrade - Job overview
Spectrum component changes for Job Overview report and tested remaining custom component.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev2Mercury\Documents\UiPath\InPwr.Bill.BillingForecast\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev5pegasus\Downloads\PADTEXT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46BFAB5C-82AF-403E-8664-DACB501D56BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54675E2D-5571-4498-9441-D8E401D8A982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -414,9 +414,6 @@
     <t>EM0002</t>
   </si>
   <si>
-    <t>mercury@inpwrinc.com;calypso@inpwrinc.com</t>
-  </si>
-  <si>
     <t>Common Utilities</t>
   </si>
   <si>
@@ -732,9 +729,6 @@
 &lt;/p&gt;</t>
   </si>
   <si>
-    <t>BillingForecast_JobQueue</t>
-  </si>
-  <si>
     <t>Percent Complete</t>
   </si>
   <si>
@@ -745,6 +739,12 @@
   </si>
   <si>
     <t>C14</t>
+  </si>
+  <si>
+    <t>BillingForecast_JobQueue_Test</t>
+  </si>
+  <si>
+    <t>mercury@inpwrinc.com;calypso@inpwrinc.com;pegasus@inpwrinc.com</t>
   </si>
 </sst>
 </file>
@@ -865,9 +865,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -877,6 +874,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1194,15 +1192,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y69"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.42578125" customWidth="1"/>
-    <col min="4" max="25" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="46.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="67.44140625" customWidth="1"/>
+    <col min="4" max="25" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="18.75">
+    <row r="1" spans="1:25" ht="18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1316,8 +1314,8 @@
       <c r="A9" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="19" t="s">
-        <v>122</v>
+      <c r="B9" s="18" t="s">
+        <v>121</v>
       </c>
       <c r="C9" t="s">
         <v>91</v>
@@ -1328,7 +1326,7 @@
         <v>64</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C10" t="s">
         <v>92</v>
@@ -1339,7 +1337,7 @@
         <v>66</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C11" t="s">
         <v>89</v>
@@ -1413,10 +1411,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>95</v>
@@ -1426,8 +1424,8 @@
       <c r="A19" t="s">
         <v>96</v>
       </c>
-      <c r="B19" s="18" t="s">
-        <v>122</v>
+      <c r="B19" s="17" t="s">
+        <v>121</v>
       </c>
       <c r="C19" t="s">
         <v>91</v>
@@ -1446,7 +1444,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B21" s="8" t="s">
         <v>67</v>
@@ -1457,24 +1455,24 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="C22" t="s">
         <v>209</v>
-      </c>
-      <c r="C22" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C23" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1485,7 +1483,7 @@
         <v>115</v>
       </c>
       <c r="C24" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1496,7 +1494,7 @@
         <v>114</v>
       </c>
       <c r="C25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1507,7 +1505,7 @@
         <v>113</v>
       </c>
       <c r="C26" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1528,299 +1526,299 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
+        <v>188</v>
+      </c>
+      <c r="B31" s="8" t="s">
         <v>189</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B40" s="7" t="s">
         <v>207</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" t="s">
+        <v>126</v>
+      </c>
+      <c r="B43" s="8" t="s">
         <v>127</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
+        <v>164</v>
+      </c>
+      <c r="B50" s="8" t="s">
         <v>165</v>
-      </c>
-      <c r="B50" s="8" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
+        <v>185</v>
+      </c>
+      <c r="B58" s="8" t="s">
         <v>186</v>
-      </c>
-      <c r="B58" s="8" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
+        <v>177</v>
+      </c>
+      <c r="B61" s="8" t="s">
         <v>178</v>
-      </c>
-      <c r="B61" s="8" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
+        <v>159</v>
+      </c>
+      <c r="B63" s="8" t="s">
         <v>160</v>
-      </c>
-      <c r="B63" s="8" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C64" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C65" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
+        <v>154</v>
+      </c>
+      <c r="B66" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="B66" s="8" t="s">
-        <v>156</v>
-      </c>
       <c r="C66" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -1833,12 +1831,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" style="8" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1875,7 +1873,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="28.8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1886,7 +1884,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -2000,7 +1998,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
+    <row r="17" spans="1:3" ht="28.8">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -2992,12 +2990,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Y966"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="32.85546875" customWidth="1"/>
-    <col min="2" max="2" width="31.140625" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="25" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="32.88671875" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" customWidth="1"/>
+    <col min="3" max="3" width="30.33203125" customWidth="1"/>
+    <col min="4" max="25" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="14.25" customHeight="1">
@@ -3043,7 +3041,7 @@
         <v>61</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>56</v>
@@ -3051,13 +3049,13 @@
     </row>
     <row r="3" spans="1:25" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C3" s="18" t="s">
         <v>122</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>121</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>65</v>
@@ -3071,7 +3069,7 @@
         <v>67</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D4" t="s">
         <v>68</v>
@@ -3085,7 +3083,7 @@
         <v>62</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D5" t="s">
         <v>63</v>
@@ -3098,14 +3096,14 @@
       <c r="B6" t="s">
         <v>94</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>122</v>
+      <c r="C6" s="17" t="s">
+        <v>121</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:25" ht="14.4">
       <c r="A7" s="12" t="s">
         <v>119</v>
       </c>
@@ -3113,7 +3111,7 @@
         <v>119</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>104</v>
@@ -3121,44 +3119,44 @@
     </row>
     <row r="8" spans="1:25" ht="14.25" customHeight="1">
       <c r="A8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="B8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1">
       <c r="A9" t="s">
+        <v>148</v>
+      </c>
+      <c r="B9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>149</v>
-      </c>
-      <c r="B9" t="s">
-        <v>149</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="14.25" customHeight="1"/>
@@ -4127,17 +4125,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A045ED-89B2-46F5-87BB-9D73B35EE197}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="18.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75">
+    <row r="1" spans="1:5" ht="18">
       <c r="A1" s="13" t="s">
         <v>42</v>
       </c>
@@ -4154,15 +4152,15 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="9" customFormat="1" ht="240">
+    <row r="2" spans="1:5" s="9" customFormat="1" ht="230.4">
       <c r="A2" s="14" t="s">
         <v>43</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="20" t="s">
-        <v>176</v>
+      <c r="C2" s="19" t="s">
+        <v>175</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>47</v>
@@ -4171,15 +4169,15 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="210">
+    <row r="3" spans="1:5" ht="201.6">
       <c r="A3" s="14" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="20" t="s">
-        <v>176</v>
+      <c r="C3" s="19" t="s">
+        <v>175</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>54</v>
@@ -4203,16 +4201,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7C6B43-6EA4-4DD0-939E-D4A6AD374EA2}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="167.5703125" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="13.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="167.5546875" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75">
+    <row r="1" spans="1:4" ht="18">
       <c r="A1" s="13" t="s">
         <v>45</v>
       </c>
@@ -4226,32 +4224,32 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="270">
+    <row r="2" spans="1:4" ht="259.2">
       <c r="A2" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="17" t="s">
-        <v>121</v>
+      <c r="B2" s="20" t="s">
+        <v>218</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="409.5">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="409.6">
       <c r="A3" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="17" t="s">
-        <v>121</v>
+      <c r="B3" s="20" t="s">
+        <v>218</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>